<commit_message>
post paul commit, getting server in line with repository
</commit_message>
<xml_diff>
--- a/data/excel_dumps/patients/patient_1.xlsx
+++ b/data/excel_dumps/patients/patient_1.xlsx
@@ -4,18 +4,18 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView activeTab="0" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible"/>
+    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
     <sheet name="Worksheet" sheetId="1" r:id="rId4"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="5">
   <si>
     <t>Student Id</t>
   </si>
@@ -30,27 +30,6 @@
   </si>
   <si>
     <t>Date</t>
-  </si>
-  <si>
-    <t>ikleiman@stonybrook.edu</t>
-  </si>
-  <si>
-    <t>false</t>
-  </si>
-  <si>
-    <t>2019-11-04</t>
-  </si>
-  <si>
-    <t>chaotsai@stonybrook.edu</t>
-  </si>
-  <si>
-    <t>2019-12-01</t>
-  </si>
-  <si>
-    <t>2019-12-03</t>
-  </si>
-  <si>
-    <t>vlgarcia@stonybrook.edu</t>
   </si>
 </sst>
 </file>
@@ -385,11 +364,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -409,147 +388,11 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2">
-        <v>6</v>
-      </c>
-      <c r="E2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3">
-        <v>2</v>
-      </c>
-      <c r="C3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3">
-        <v>10</v>
-      </c>
-      <c r="E3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="C4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4">
-        <v>7</v>
-      </c>
-      <c r="E4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="C5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5">
-        <v>32</v>
-      </c>
-      <c r="E5" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
-      <c r="A6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6">
-        <v>2</v>
-      </c>
-      <c r="C6" t="s">
-        <v>6</v>
-      </c>
-      <c r="D6">
-        <v>55</v>
-      </c>
-      <c r="E6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
-      <c r="A7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7">
-        <v>2</v>
-      </c>
-      <c r="C7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7">
-        <v>8</v>
-      </c>
-      <c r="E7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8">
-        <v>1</v>
-      </c>
-      <c r="C8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D8">
-        <v>7</v>
-      </c>
-      <c r="E8" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="A9" t="s">
-        <v>11</v>
-      </c>
-      <c r="B9">
-        <v>2</v>
-      </c>
-      <c r="C9" t="s">
-        <v>6</v>
-      </c>
-      <c r="D9">
-        <v>10</v>
-      </c>
-      <c r="E9" t="s">
-        <v>10</v>
-      </c>
-    </row>
   </sheetData>
   <sheetProtection sheet="false" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>
   <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1"/>
+  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
   <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
     <oddHeader/>
     <oddFooter/>

</xml_diff>